<commit_message>
B&N rev7 final: Paso 12 applied (9 CORREGIR, 57 rows with destination, RFI-38..53), back-check comments resolved, all gates OK; skill v80n
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/FINAL_FOR_REVIEW_2026-10-24_rev7/Take-off/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev7.xlsx
+++ b/cache_proyectos/barnes_noble/FINAL_FOR_REVIEW_2026-10-24_rev7/Take-off/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev7.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="701">
   <si>
     <t xml:space="preserve">Barnes &amp; Noble - Colorado Springs, CO (3173 Cinema Point)   |   METAL FRAMING &amp; DRYWALL TAKEOFF</t>
   </si>
@@ -154,7 +154,7 @@
     <t xml:space="preserve">Joint compound (lb per SF)</t>
   </si>
   <si>
-    <t xml:space="preserve">YIELD: 72 lb per 1,000 SF, level 4 (estimator criterion).</t>
+    <t xml:space="preserve">YIELD: 72 lb per 1,000 SF; Level 4 finish printed on A-001A Div 09 A.8 "PROVIDE AT A MINIMUM A LEVEL 4 FINISH".</t>
   </si>
   <si>
     <t xml:space="preserve">Joint tape (LF per SF)</t>
@@ -1150,7 +1150,7 @@
     <t xml:space="preserve">PCS</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: 5/A-410, 7/A-210 | Breakdown [DERIVED]: CLIP-ANGLES-5-A410 2,518 + CLIP-ANGLES-7-A210 4 = 2,522 PCS | 2" x 2" 16 GA. CLIP ANGLE at each stud per bracing row, (4) TEK SCREWS (5/A-410): rows x studs = W2-01 6x38 + W2-02 6x5 + W2-03 6x72 + W2-04 6x44 + W2-05 6x11 + W2-06.1 6x7 + W2-06.2 6x3 + W2-06.3 6x5 + W2-06.4 6x3 + W2-06.5 6x10 + W2-07 6x7 + W2-08 6x11 + W2-09 6x11 + W5-01 6x6 + W3-01 1x4 + W3-02 1x10 + W3-05 1x4 + W3-03 1x10 + W3-06 1x4 + W3-04 1x4 + W4-28a 1x8 + W4-28b 1x3 + W4-28c 1x3 + W4-28d 1x3 + W4-28e 1x3 + W4-29a 1x5 + W4-29b 1x5 + W4-29c 1x5 + W4-29d 1x5 + W4-29e 1x5 + W4-29f 1x5 + W4-30a 1x5 + W4-30b 1x5 + W4-30c 1x5 + W4-30d 1x5 + W4-30e 1x5 + W4-30f 1x5 + W4-31a 1x8 + W4-31b 1x3 + W4-31c 1x3 + W4-31d 1x3 + W4-31e 1x3 + CW-01 1x12 + CW-02 1x12 + CW-03 1x12 + CW-04 1x12 + CW-05 </t>
+    <t xml:space="preserve">N/SHEET: 5/A-410, 7/A-210 | Breakdown [DERIVED]: CLIP-ANGLES-5-A410 2,518 + CLIP-ANGLES-7-A210 4 = 2,522 PCS | 2" x 2" 16 GA. CLIP ANGLE at each stud per bracing row, (4) TEK SCREWS (5/A-410): rows x studs = W2-01 6x38 + W2-02 6x5 + W2-03 6x72 + W2-04 6x44 + W2-05 6x11 + W2-06.1 6x7 + W2-06.2 6x3 + W2-06.3 6x5 + W2-06.4 6x3 + W2-06.5 6x10 + W2-07 6x7 + W2-08 6x11 + W2-09 6x11 + W5-01 6x6 + W3-01 1x4 + W3-02 1x10 + W3-05 1x4 + W3-03 1x10 + W3-06 1x4 + W3-04 1x4 + W4-28a 1x8 + W4-28b 1x3 + W4-28c 1x3 + W4-28d 1x3 + W4-28e 1x3 + W4-29a 1x5 + W4-29b 1x5 + W4-29c 1x5 + W4-29d 1x5 + W4-29e 1x5 + W4-29f 1x5 + W4-30a 1x5 + W4-30b 1x5 + W4-30c 1x5 + W4-30d 1x5 + W4-30e 1x5 + W4-30f 1x5 + W4-31a 1x8 + W4-31b 1x3 + W4-31c 1x3 + W4-31d 1x3 + W4-31e 1x3 + CW-01 1x12 + CW-02 1x12 + CW-03 1x12 + CW-04 1x12 + CW-05 1x12 + CW-06 1x12 + CW-07 1x12 + CW-08 1x12 + CW-09 1x12 + C-H1-N 6x24 + C-H1-W 6x11 + C-H2a 6x11 + C-H2b 6x3 + C-H3a 6x5 + C-H3b 6x6 + C-E2 6x23 + C-E1-S 6x19 + C-I-P.1 6x2 + C-E1-P.2 6x3 + C-E1-B 6x3 + C-F 6x4 + C-I 6x3 + SS-N 3x19 + SS-E 3x9 + SS-IN-N 3x16 + SS-IN-E 3x6 + SS-GG 4x6 = 2518 pcs; 3"x3"x16 GA. CLIP ANGLES at the nested header to jamb connection (7/A-210): 2 header ends x 2 (front / back) = 4 pcs (conservative; count not printed - RFI-51)</t>
   </si>
   <si>
     <t xml:space="preserve">X-EDNI fasteners 0.145" (Hilti), top track to structure (A-410 note 8.C)</t>
@@ -1258,7 +1258,7 @@
     <t xml:space="preserve">PVC trim - edge trim molding and inside corner molding at the FRP</t>
   </si>
   <si>
-    <t xml:space="preserve">[DERIVED] N/SHEET: A-510, A-225 | none: FRP-1 (A-510: Cafe Work Room 104 walls, Janitor 107 walls, Cafe 103 below countertop) - no FRP height / extent printed for partitions (A-225 finish plan dashed FRP-1 zones only) - not quantified, RFI-13 with delta</t>
+    <t xml:space="preserve">[DERIVED] N/SHEET: 4/A-226B, 12/A-200 | none: FRP-1 (A-510): Cafe Work Room 104 FRP-1 full height to the 10'-0" ceiling (1-4/A-226B); Janitor 107 FRP-1 to 96" A.F.F. (A-131) / 8'-0" (9-12/A-200); Cafe 103 below countertop. Installer not defined (A-002) - not carried, RFI-13 with delta (1,030.64 SF) - PVC trim with it.</t>
   </si>
   <si>
     <t xml:space="preserve">Power-driven fasteners and duct sleeves</t>
@@ -1360,7 +1360,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-24 (rev1): perimeter walls types 1 / 1A / 1B / 1C are EXISTING (1/DM-101 legend solid = to remain + key note 3 "EXTERIOR WALL PATCH AND REPAIR AS REQUIRED TO MAINTAIN EXISTING FIRE RATING"; A-101 Construction Legend "EXISTING EXTERIOR WALL" / "EXISTING PARTITION"; A-002 "PERIMETER STUDS, INSULATION, VAPOR BARRIER F/I BY LL"). Perimeter framing (studs, track, bracing, 1B sheathing) EXCLUDED. Interior face patch &amp; repair (1/DM-101 key note 3, A-101 C5) = ALLOWANCE, amount: $ ________ (blank, estimator to fill). rev2 (estimator decision 2026-10-25): break room kitchenette W.R. on existing EXT-07 (6/A-412, 7/A-412) is INSIDE this patch &amp; repair allowance; allowance amount stays BLANK (decided). Paso 12 (rev7): A-410 types 1, 1A, 1B, 1C label the interior board "5/8" GYP BD BY FUTURE TENANT": EXCLUDED with that citation, consistent with this decision. A-413 7/8A general note "IF SHELVING IS TO BE INSTALLED ON EXISTING WALL, G.C. IS TO REMOVE AND REPLACE GYP. BOARD AS REQUIRED FOR INSTALLATION OF WOOD BLOCKING": inside this patch &amp; repair allowance.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied: - 417.43 LF of perimeter walls (17 walls); 3-5/8" stud 16,812.96 -&gt; 10,120.39 LF; 8" stud 2,332.99 -&gt; 0; 1/2" exterior sheathing 2,469.22 -&gt; 0 SF; bottom / top track 1,051.87 -&gt; 634.44 LF each; bracing 5,230.74 -&gt; 2,827.81 LF. Allowance: blank.</t>
+    <t xml:space="preserve">Applied: - 417.43 LF of perimeter walls (17 walls); 3-5/8" stud 16,812.96 -&gt; 10,120.39 LF; 8" stud 2,332.99 -&gt; 0; 1/2" exterior sheathing 2,469.22 -&gt; 0 SF; bottom / top track 1,051.87 -&gt; 634.44 LF each; bracing 5,230.74 -&gt; 2,827.81 LF. Allowance: blank.; board by future tenant on the existing perimeter (A-410 types 1 / 1A / 1B / 1C): upper bound 417.43 LF x 25.0 = 10,436 SF 5/8" Type X if it were ever in our scope.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-02</t>
@@ -1384,10 +1384,10 @@
     <t xml:space="preserve">RFI-04</t>
   </si>
   <si>
-    <t xml:space="preserve">CLOSED - Review Item rev3 (estimator decision 2026-10-26): type 2 &gt; 22 ft: 3-5/8" 14 ga SJ + diagonal braces @ 32" O.C. to structure (3/A-410 "PROVIDE DIAGONAL BRACING AT 32" O.C. TO STRUCTURE (TYP.)"); brace member / length not printed - estimator choice 3-5/8" 20 ga stud x 4 ft at 45 deg. Paso 12 (rev7): same precedent applied to the Cafe 3-5/8" walls to deck (C-H2a, C-H2b, C-F): 14 ga SJ + 11 diagonal braces = 44.0 LF.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Applied: 117 braces (115 in rev2 + 2 from W2-05 +5.00 LF) x 4.0 ft = 468.0 LF 3-5/8" 20 ga stud (DERIVED, member and length = estimator choice; note kept). Citation corrected: diagonal bracing is on 3/A-410 Top Track Detail (rev0-rev2 said 3/A-410).</t>
+    <t xml:space="preserve">CLOSED - Review Item rev3 (estimator decision 2026-10-26): type 2 &gt; 22 ft: 3-5/8" 14 ga SJ + diagonal braces @ 32" O.C. to structure (3/A-410 Top Track Detail "PROVIDE DIAGONAL BRACING AT 32" O.C. TO STRUCTURE ABOVE (TYP.)"); brace member / length not printed - estimator choice 3-5/8" 20 ga stud x 4 ft at 45 deg. Paso 12 (rev7): same precedent applied to the Cafe 3-5/8" walls to deck (C-H2a, C-H2b, C-F): 14 ga SJ + 11 diagonal braces = 44.0 LF.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied: 117 braces x 4.0 ft = 468.0 LF (type 2) + 44.0 LF (Cafe) 3-5/8" 20 ga stud (member and length = estimator choice). Citation history: rev0-rev2 cited the partition type 3 section, rev3-rev6 cited 8/A-410 (that bubble is the Typ. Connection Detail); the Top Track Detail is bubble 3/A-410 (Paso 12 C-07).</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-05</t>
@@ -1405,7 +1405,7 @@
     <t xml:space="preserve">CLOSED - Review Item rev3 (estimator decision 2026-10-26): Cafe walls H1, H2a, H2b, H3a, H3b, F studs TO DECK 25'-0" (1/A-400B draws the Cafe walls floor to B.O. DECK; A-226A elevations break at the top; no section prints a stud top). Board per face = ceiling + 6" (A-410 partition note 3): Workroom ACT-1 10'-0" -&gt; 10'-6"; Grab &amp; Go GWB 7'-1" -&gt; 7'-7"; Cafe open-to-deck strip at H2a (1/A-121 PT-6 OPEN TO DECK) -&gt; to deck.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied (faces already at these heights in rev2;.</t>
+    <t xml:space="preserve">Applied (faces already at these heights in rev2; RCP evidence on 1/A-121).</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-07</t>
@@ -1444,7 +1444,7 @@
     <t xml:space="preserve">CLOSED - estimator decision RFI-11 (rev1) + plan check rev6: W.R. gypsum board on all faces of Women's 109, Men's 108, Janitor 107 and the drinking fountain alcove (A-410 Partition Notes 2 "PROVIDE WATER RESISTANT GYPSUM BOARD IN ALL BATHROOMS AND JANITOR'S CLOSET FOR WALL AND CEILING CONSTRUCTION", note 7, "*" note, 2/A-410, 5/A-410; A-001A Div 09 A.4) and on the restroom GWB ceilings (same note 2; 1/A-121 GWB 9'-0"). Cafe Work Room 104: NO W.R. - G/A-221 draws only 5/8" FRT plywood on the Work Room side (FRP-1 finish, A-510); there is no gypsum board on that face (rev6 removes the 570.36 SF GWB faces).</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied (rev6): 5/8" Type X W.R. = 1,092.59 SF = walls (Women's 222.93 + Men's 223.02 + Janitor 485.75 + alcove corridor 88.63) + restroom ceilings 122.30 (Women's 61.19 + Men's 61.11, 1/A-121).</t>
+    <t xml:space="preserve">Applied (rev7): 5/8" Type X W.R. = 1,092.59 SF = walls (Women's 222.93 + Men's 223.02 + Janitor 485.75 + alcove corridor 88.63) + restroom ceilings 122.30 - 1'-2" cement board base 50.04 (22/A-201).</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-12</t>
@@ -1549,7 +1549,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-24 (rev1): FRT blocking taken off with the counts and rows per detail: stock room shelving 7/A-413 (3 rows), receiving table 8A/A-413 (4 rows), Manager's Office 3, 4/A-412 (4 rows), break room cabinets 6/A-412 (2 rows); restroom backing 21, 26/A-201 (10 pcs 3/4" FRT plywood); Cafe menu boards 4/A-226A continuous 3/4" FRT plywood 31" high x C-E1-S.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied: FRT blocking 585.27 LF (387.0 + 69.0 + 85.6 + 10.67); 3/4" FRT plywood + 60.61 SF menu boards (23.46 x 31/12) + 17.78 SF restroom backing (10 pcs x 16" bay x 16" high, rev2 (estimator decision 2026-10-25): 13.33 x 16/12). rev5: water heater backing (P-201) carried conservatively -&gt; RFI-32; janitor 3/4" FRT plywood area (11/A-200) carried 17.0 SF -&gt; RFI-33; W-3 surface blocking (1/A-414, 7/A-414) -&gt; RFI-36.</t>
+    <t xml:space="preserve">Applied: FRT blocking 585.27 LF (387.0 + 69.0 + 85.6 + 10.67 + FE cabinets 16.0, rev7); 3/4" FRT plywood + 60.61 SF menu boards (23.46 x 31/12) + 17.78 SF restroom backing (10 pcs x 16" bay x 16" high, rev2 (estimator decision 2026-10-25): 13.33 x 16/12). rev5: water heater backing (P-201) carried conservatively -&gt; RFI-32; janitor 3/4" FRT plywood area (11/A-200) carried 17.0 SF -&gt; RFI-33; W-3 surface blocking (1/A-414, 7/A-414) -&gt; RFI-36.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-24</t>
@@ -1582,7 +1582,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-24 (rev1): all 5/8" gyp bd on new walls AND GWB ceilings = Type X (A-001A Div 09 A.2; 4/A-121, 5/A-121 - rev2 (estimator decision 2026-10-25): ceilings to Type X); W.R. faces = 5/8" Type X W.R. No 5/8" regular remains.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied (rev6): 5/8" Type X 15,109.29 SF = walls 14,100.86 + GWB ceilings 884.24 (restroom ceilings moved to W.R., RFI-11) + vestibule box 105.5 + Grab &amp; Go soffit bottom 3.73; Type X W.R. 1,092.59 SF; 5/8" regular 0.</t>
+    <t xml:space="preserve">Applied (rev7): 5/8" Type X 15,109.29 SF = walls 14,100.86 + GWB ceilings 884.24 (Cafe 103 - 11'-6" GWB band 125.07, Cafe 103 - 9'-0" GWB band 50.67, Cafe Seating Area 102 - GWB cloud 573.69, Cafe 103 - 11'-0" GWB zone 109.65, Grab &amp; Go 25.16) + VEST-GWB 105.5 + SS-GG-BOTTOM-GWB 3.73 + VEST-GWB-BANDS 14.96; Type X W.R. 1,092.59 SF; 5/8" regular 0.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-28</t>
@@ -1651,7 +1651,7 @@
     <t xml:space="preserve">RFI-35</t>
   </si>
   <si>
-    <t xml:space="preserve">3/A-410 Top Track Detail "METAL STUD/TRACK FIRE STOP AT CEILING LINE, TYP." (citation corrected from 3/A-410 - Paso 12 (rev7): C-07): applied to every full-height wall with a ceiling on at least one face (1/A-121); carried; confirm with the GC.</t>
+    <t xml:space="preserve">3/A-410 Top Track Detail "METAL STUD/TRACK FIRE STOP AT CEILING LINE, TYP." (rev5-rev6 cited 8/A-410, which is the Typ. Connection Detail - Paso 12 C-07): applied to every full-height wall with a ceiling on at least one face (1/A-121); carried; confirm with the GC.</t>
   </si>
   <si>
     <t xml:space="preserve">Carried per wall (Material Summary breakdown) = 264.21 LF; if not required: minus that LF.</t>
@@ -1792,13 +1792,31 @@
     <t xml:space="preserve">Carried 32.0 SF 3/4" FRT plywood; if by the electrical contractor: - 32.0 SF.</t>
   </si>
   <si>
+    <t xml:space="preserve">RFI-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vestibule GWB bands above B.O. ceiling 10'-6": top of the band 11'-3 1/2" V.I.F. (2/A-210, 3/A-210, "VESTIBULE ASSEMBLY TO MATCH EXISTING STOREFRONT SYSTEM V.I.F.").</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carried 14.96 SF; each 1" of band height = 1.89 SF (front 12.67 + sides 2 x 8.42 ft / 12).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFI-53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Light fixtures in the Cafe GWB bands (11'-6" and 9'-0", 1/A-121): fixture count in the bands not taken; 5/A-121 "PROVIDE ADDITIONAL WIRE SUPPORT AT ALL LIGHT FIXTURES".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each fixture in a band = + 1 hanger x 13.5 / 16.0 ft wire.</t>
+  </si>
+  <si>
     <t xml:space="preserve">RFI-51</t>
   </si>
   <si>
     <t xml:space="preserve">Fastener counts not printed: 7/A-210 3"x3"x16 ga clip angles (count per header end); cement board screw spacing (manufacturer standard 8" O.C. used); plywood screws per A-410 note 8.D (24" field / 12" perimeter on 4x8 sheets).</t>
   </si>
   <si>
-    <t xml:space="preserve">Carried: clip angles 7/A-210 4 pcs; cement board screws 1686 pcs; plywood screws 2331 pcs - adjust to the estimator yields.</t>
+    <t xml:space="preserve">Carried: clip angles 7/A-210 4 pcs; cement board screws 1686 pcs; plywood screws 2331 pcs - adjust to the estimator yields. Framing screws count the stud pieces of the walls and column wraps (781); the detail members (braces, cross members, posts, bracing) add about + 724 screws. Slab pins at 12" O.C. (estimator criterion); A-410 note 8.F (2 rows at 16" O.C. into concrete) = about + 321 pins.</t>
   </si>
   <si>
     <t xml:space="preserve">0 questions in total, asked ONE at a time in this order: floor plan (partition types A-Z), then the details the floor plan calls, in order</t>
@@ -1933,7 +1951,7 @@
     <t xml:space="preserve">Gypsum board ceilings</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantified (rev6): suspended GWB ceilings and soffits per A-121 (5/A-121, 4/A-121) and 2/A-221 = 981.38 SF: 5/8" Type X 884.24 SF + restroom ceilings 5/8" Type X W.R. 122.30 SF (A-410 Partition Notes 2).</t>
+    <t xml:space="preserve">Quantified (rev7): suspended GWB ceilings and soffits per A-121 (5/A-121, 4/A-121) and 2/A-221 = 1,006.54 SF (incl. Grab &amp; Go 7'-1" 25.16 SF): 5/8" Type X + restroom ceilings 5/8" Type X W.R. (A-410 Partition Notes 2).</t>
   </si>
   <si>
     <t xml:space="preserve">ALC-12</t>
@@ -1942,7 +1960,7 @@
     <t xml:space="preserve">Ceiling suspension (furring / carrying channel / hanger wire / ceiling track)</t>
   </si>
   <si>
-    <t xml:space="preserve">Furring channel @ 24", carrying channel @ 48", hanger wire 103 pcs, ceiling track per 5/A-121 on A-121; carrying direction E-W (RFI-15 CLOSED rev3: joists N-S on 1/A-400A, 2/A-400A); Cafe Seating cloud = USG drywall suspension grid 4/A-121; M-100 (p46), M-101 (p47), M-102 (p48) hangers are MEP; Grab &amp; Go GWB ceiling 7'-1" added; additional hangers at light fixtures and seismic splay wires per 5/A-121 (RFI-38); 16 ga tie wire (5/A-121) = consumable of the furring / carrying install, no separate row.</t>
+    <t xml:space="preserve">Furring channel @ 24", carrying channel @ 48", hanger wire 109 pcs at 48" + 29 at light fixtures, ceiling track per 5/A-121 on A-121; carrying direction E-W (RFI-15 CLOSED rev3: joists N-S on 1/A-400A, 2/A-400A); Cafe Seating cloud = USG drywall suspension grid 4/A-121; M-100 (p46), M-101 (p47), M-102 (p48) hangers are MEP; Grab &amp; Go GWB ceiling 7'-1" added; additional hangers at light fixtures and seismic splay wires per 5/A-121 (RFI-38); 16 ga tie wire (5/A-121) = consumable of the furring / carrying install, no separate row.</t>
   </si>
   <si>
     <t xml:space="preserve">ALC-13</t>
@@ -1978,7 +1996,7 @@
     <t xml:space="preserve">Blocking (FRT wood / metal) for millwork and accessories</t>
   </si>
   <si>
-    <t xml:space="preserve">Quantified (rev1, RFI-23): FRT blocking 585.27 LF (7/A-413 387.0, 8A/A-413 69.0, 3-4/A-412 85.6, 6/A-412 10.67) + 3/4" FRT plywood menu boards 60.61 SF (4/A-226A) + restroom backing 17.78 SF (21/A-201) + janitor 17.0 SF (11/A-200, RFI-33); water heater backing P-201 10.67 LF 3-5/8" stud (RFI-32); W-3 surface blocking 1/A-414 RFI-36.</t>
+    <t xml:space="preserve">Quantified (rev1, RFI-23): FRT blocking 585.27 LF (7/A-413 387.0, 8A/A-413 69.0, 3-4/A-412 85.6, 6/A-412 10.67, 4/A-101 FE cabinets 16.0) + 2X wood 17.0 LF (2/A-500) + 3/4" FRT plywood menu boards 60.61 SF (4/A-226A) + restroom backing 17.78 SF (21/A-201) + janitor 17.0 SF (11/A-200, RFI-33); water heater backing P-201 10.67 LF 3-5/8" stud (RFI-32); W-3 surface blocking 1/A-414 RFI-36.</t>
   </si>
   <si>
     <t xml:space="preserve">ALC-17</t>
@@ -2053,7 +2071,7 @@
     <t xml:space="preserve">QUANTIFIED: Level 4 finish printed - A-001A Div 09 A.8 "PROVIDE AT A MINIMUM A LEVEL 4 FINISH" (joint compound / tape yields per Inputs); no Level 5 (A-510).</t>
   </si>
   <si>
-    <t xml:space="preserve">ALC-X26</t>
+    <t xml:space="preserve">ALC-X40</t>
   </si>
   <si>
     <t xml:space="preserve">Acoustical lay-in ceilings ACT-1 / ACT-3 (tile + Prelude XL grid + wires)</t>
@@ -2062,7 +2080,7 @@
     <t xml:space="preserve">EXCLUDED: Div 09 51 acoustical ceilings by the ACT contractor - A-002 lists "ACOUSTICAL CEILING SYSTEM" as its own line (F/I tenant contractor); ACT-1 Cafe Workroom 10'-0", ACT-3 Corridor, Break Room, Manager's Office 9'-0" (1/A-121, A-510 finish legend); ACT portion of 5/A-121. Wall board heights use these ceilings + 6".</t>
   </si>
   <si>
-    <t xml:space="preserve">ALC-X27</t>
+    <t xml:space="preserve">ALC-X41</t>
   </si>
   <si>
     <t xml:space="preserve">Unistrut space frame / strut channel</t>
@@ -2071,7 +2089,7 @@
     <t xml:space="preserve">EXCLUDED: A-001A Div 05 D "UNISTRUT SPACE FRAME GRID SYSTEM ... AS REQUIRED FOR LIGHTING, CEILING ACCESSORIES OR MECHANICAL SYSTEMS SUSPENSION" and A-002 cafe signage "STRUT CHANNEL" = lighting / sign / MEP supports by those trades; the sign blocking is carried (4/A-226A menu boards).</t>
   </si>
   <si>
-    <t xml:space="preserve">ALC-X28</t>
+    <t xml:space="preserve">ALC-X42</t>
   </si>
   <si>
     <t xml:space="preserve">Caulk at the base of wet-area walls</t>
@@ -2080,7 +2098,7 @@
     <t xml:space="preserve">EXCLUDED: A-101 general note 8 "BOTTOM OF THE WALL CAULKED AT FLOOR LEVEL" = joint sealant (Div 07), excluded like all sealants (estimator standing order).</t>
   </si>
   <si>
-    <t xml:space="preserve">ALC-X29</t>
+    <t xml:space="preserve">ALC-X43</t>
   </si>
   <si>
     <t xml:space="preserve">Partition seismic bracing (A-002 Div 10)</t>
@@ -2089,15 +2107,18 @@
     <t xml:space="preserve">EXCLUDED as a separate item: A-002 Div 10 "SEISMIC BRACING" is listed with the specialties; partition lateral bracing is carried per 5/A-410 and 3/A-410; ceiling bracing per 5/A-121 carried under RFI-38.</t>
   </si>
   <si>
+    <t xml:space="preserve">ALC-X44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remove &amp; replace existing GWB for shelving blocking (7/A-413)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inside the RFI-01 patch &amp; repair allowance (existing perimeter walls): A-413 general note "G.C. IS TO REMOVE AND REPLACE GYP. BOARD AS REQUIRED FOR INSTALLATION OF WOOD BLOCKING".</t>
+  </si>
+  <si>
     <t xml:space="preserve">ALC-X30</t>
   </si>
   <si>
-    <t xml:space="preserve">Remove &amp; replace existing GWB for shelving blocking (7/A-413)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inside the RFI-01 patch &amp; repair allowance (existing perimeter walls): A-413 general note "G.C. IS TO REMOVE AND REPLACE GYP. BOARD AS REQUIRED FOR INSTALLATION OF WOOD BLOCKING".</t>
-  </si>
-  <si>
     <t xml:space="preserve">batt insulation</t>
   </si>
   <si>
@@ -2107,7 +2128,7 @@
     <t xml:space="preserve">reglas.py compuerta OK</t>
   </si>
   <si>
-    <t xml:space="preserve">{"canon": "a2b1eb953623f091c459cd5e3649f888037ba01214e1bad07e2cb3d6ae03246f", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "2595754ec20f9e38b1232226d0f9fe68e8995a81448a9ce869d3943eb01fc81c", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
+    <t xml:space="preserve">{"canon": "47198641f746c0c3aaff104d86c478b8629dfe00c16faed73946af08016d7263", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "943ff7bb50599871e6bbd3e4d57748b5c9338105b4ae26b344d45f16d0214ea4", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
   </si>
 </sst>
 </file>
@@ -7325,7 +7346,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
@@ -7924,6 +7945,28 @@
       </c>
       <c r="C54" s="0" t="s">
         <v>590</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="0" t="s">
+        <v>591</v>
+      </c>
+      <c r="B55" s="0" t="s">
+        <v>592</v>
+      </c>
+      <c r="C55" s="0" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="0" t="s">
+        <v>594</v>
+      </c>
+      <c r="B56" s="0" t="s">
+        <v>595</v>
+      </c>
+      <c r="C56" s="0" t="s">
+        <v>596</v>
       </c>
     </row>
   </sheetData>
@@ -7955,27 +7998,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
     </row>
   </sheetData>
@@ -8005,436 +8048,436 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>59</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>433</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="C18" s="0" t="s">
         <v>433</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="C30" s="0" t="s">
         <v>433</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>687</v>
+        <v>696</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
     </row>
   </sheetData>
@@ -8458,12 +8501,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>692</v>
+        <v>699</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>